<commit_message>
working scm model, adapted the evg sink distances based on centroid
</commit_message>
<xml_diff>
--- a/NG_flows_scm.xlsx
+++ b/NG_flows_scm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/scm_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{063E1CBA-981A-4F9C-9ABC-D9966DC7B63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6A831B4-8A3D-4FBB-ABB4-2198D55885D9}"/>
+  <xr:revisionPtr revIDLastSave="25" documentId="8_{063E1CBA-981A-4F9C-9ABC-D9966DC7B63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E77FD392-8979-4E08-976D-874911313D3A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{3FD26122-B3FE-4856-AD14-3A87BCC0C804}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{3FD26122-B3FE-4856-AD14-3A87BCC0C804}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="44">
   <si>
     <t>year</t>
   </si>
@@ -194,16 +194,20 @@
   <si>
     <t>supply_fraction</t>
   </si>
+  <si>
+    <t>Transport</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="#,##0.##########"/>
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -273,6 +277,33 @@
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="161"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -424,11 +455,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -482,8 +524,13 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="9">
+    <cellStyle name="Komma 2" xfId="7" xr:uid="{A73D8BCA-A881-4B1C-AF23-3AF20EC5833F}"/>
     <cellStyle name="Link" xfId="2" builtinId="8"/>
+    <cellStyle name="Normal 2" xfId="4" xr:uid="{D20AB9E2-2957-4169-9AF8-2BB039F9A456}"/>
+    <cellStyle name="Normal 4" xfId="8" xr:uid="{2E1E22F4-38B9-423B-B1D4-F42DFC421E62}"/>
+    <cellStyle name="Notes" xfId="5" xr:uid="{47C33B30-13B4-4A20-A565-7A5B4FBED5D0}"/>
+    <cellStyle name="Notes 3" xfId="6" xr:uid="{12128CAA-9CBF-4230-9565-27E9BF4B9B26}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="1" xr:uid="{8F10BC5A-D3E5-4B64-83C5-D986D807AE23}"/>
     <cellStyle name="Standard 3" xfId="3" xr:uid="{356112E7-E834-4F9F-A0C5-FB9E132175AA}"/>
@@ -873,7 +920,6 @@
         <v>5</v>
       </c>
       <c r="D2" s="2">
-        <f>28/3.6</f>
         <v>7.7777777777777777</v>
       </c>
     </row>
@@ -888,7 +934,6 @@
         <v>6</v>
       </c>
       <c r="D3" s="2">
-        <f>2.67</f>
         <v>2.67</v>
       </c>
     </row>
@@ -903,7 +948,6 @@
         <v>7</v>
       </c>
       <c r="D4" s="2">
-        <f>(27+10)/1000</f>
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
@@ -912,14 +956,13 @@
         <v>2025</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D5" s="2">
-        <f>108002.01194/1000</f>
-        <v>108.00201194</v>
+        <v>1.1111111111111112</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
@@ -930,11 +973,10 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2">
-        <f>92367.37174/1000</f>
-        <v>92.367371739999996</v>
+        <v>68.366</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.25">
@@ -945,11 +987,10 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="2">
-        <f>(306984.86711+84484.70625)/1000</f>
-        <v>391.46957335999997</v>
+        <v>192.197</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.25">
@@ -957,14 +998,13 @@
         <v>2025</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2">
-        <f>76029.7465155539*0.01163</f>
-        <v>884.2259519758918</v>
+        <v>346.64400000000001</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.25">
@@ -972,14 +1012,13 @@
         <v>2025</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D9" s="2">
-        <f>(512731.305090136+32085+13246)/1000</f>
-        <v>558.06230509013596</v>
+        <v>2.113</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -990,26 +1029,24 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D10" s="2">
-        <f>((4779+64753)+(1341+33309))*0.01163</f>
-        <v>1211.6366599999999</v>
+        <v>884.2259519758918</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>2030</v>
+        <v>2025</v>
       </c>
       <c r="B11" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2">
-        <f>21.5/3.6</f>
-        <v>5.9722222222222223</v>
+        <v>558.06230509013596</v>
       </c>
       <c r="L11" s="16">
         <v>2024</v>
@@ -1021,16 +1058,16 @@
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>2030</v>
+        <v>2025</v>
       </c>
       <c r="B12" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D12" s="2">
-        <v>2.14</v>
+        <v>1140.4610599999999</v>
       </c>
       <c r="L12" s="19"/>
       <c r="M12" s="20" t="s">
@@ -1048,16 +1085,16 @@
     </row>
     <row r="13" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>2030</v>
+        <v>2025</v>
       </c>
       <c r="B13" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2">
-        <v>0</v>
+        <v>37.147113297707328</v>
       </c>
       <c r="L13" s="22" t="s">
         <v>9</v>
@@ -1084,14 +1121,13 @@
         <v>2030</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="2">
-        <f>83808.51264/1000</f>
-        <v>83.808512640000004</v>
+        <v>5.9722222222222223</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
@@ -1099,14 +1135,13 @@
         <v>2030</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="2">
-        <f>59066.88433/1000</f>
-        <v>59.066884330000001</v>
+        <v>2.14</v>
       </c>
       <c r="G15" t="s">
         <v>30</v>
@@ -1137,14 +1172,13 @@
         <v>2030</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C16" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="2">
-        <f>(304612.30516+74920.18644)/1000</f>
-        <v>379.53249160000001</v>
+        <v>0</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>17</v>
@@ -1218,14 +1252,13 @@
         <v>2030</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D17" s="2">
-        <f>59349.0264746045*0.01163</f>
-        <v>690.22917789965027</v>
+        <v>2.2222222222222223</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>28</v>
@@ -1299,14 +1332,13 @@
         <v>2030</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" s="2">
-        <f>(436539+21487+8798)/1000</f>
-        <v>466.82400000000001</v>
+        <v>83.808512640000004</v>
       </c>
       <c r="G18" t="s">
         <v>4</v>
@@ -1378,14 +1410,13 @@
         <v>2030</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="2">
-        <f>((2365+38938)+(561+17215))*0.01163</f>
-        <v>687.08876999999995</v>
+        <v>59.066884330000001</v>
       </c>
       <c r="G19" t="s">
         <v>8</v>
@@ -1453,18 +1484,17 @@
       </c>
     </row>
     <row r="20" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A20" s="3">
-        <v>2035</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>5</v>
+      <c r="A20">
+        <v>2030</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
       </c>
       <c r="D20" s="2">
-        <f>15/3.6</f>
-        <v>4.166666666666667</v>
+        <v>379.53249160000001</v>
       </c>
       <c r="G20" t="s">
         <v>11</v>
@@ -1521,17 +1551,17 @@
       <c r="AB20" s="11"/>
     </row>
     <row r="21" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A21" s="3">
-        <v>2035</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>6</v>
+      <c r="A21">
+        <v>2030</v>
+      </c>
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" t="s">
+        <v>43</v>
       </c>
       <c r="D21" s="2">
-        <v>1.6</v>
+        <v>1.2689999999999999</v>
       </c>
       <c r="G21" t="s">
         <v>39</v>
@@ -1598,17 +1628,17 @@
       </c>
     </row>
     <row r="22" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="3">
-        <v>2035</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>7</v>
+      <c r="A22">
+        <v>2030</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
+        <v>5</v>
       </c>
       <c r="D22" s="2">
-        <v>0</v>
+        <v>690.22917789965027</v>
       </c>
       <c r="G22" t="s">
         <v>33</v>
@@ -1674,18 +1704,17 @@
       <c r="AB22" s="4"/>
     </row>
     <row r="23" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="3">
-        <v>2035</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>5</v>
+      <c r="A23">
+        <v>2030</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
       </c>
       <c r="D23" s="2">
-        <f>49879.76929/1000</f>
-        <v>49.879769289999999</v>
+        <v>466.82400000000001</v>
       </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
@@ -1710,18 +1739,17 @@
       <c r="AB23" s="4"/>
     </row>
     <row r="24" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="3">
-        <v>2035</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>6</v>
+      <c r="A24">
+        <v>2030</v>
+      </c>
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
       </c>
       <c r="D24" s="2">
-        <f>58785.07618/1000</f>
-        <v>58.785076179999997</v>
+        <v>653.05939000000001</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>31</v>
@@ -1749,18 +1777,17 @@
       <c r="AB24" s="4"/>
     </row>
     <row r="25" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="3">
-        <v>2035</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>7</v>
+      <c r="A25">
+        <v>2030</v>
+      </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>43</v>
       </c>
       <c r="D25" s="2">
-        <f>(231931.47942+63918.38921)/1000</f>
-        <v>295.84986863</v>
+        <v>70.128610870803428</v>
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
@@ -1789,14 +1816,13 @@
         <v>2035</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D26" s="2">
-        <f>44288.3805839263*0.01163</f>
-        <v>515.07386619106285</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="G26" t="s">
         <v>32</v>
@@ -1830,14 +1856,13 @@
         <v>2035</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="2">
-        <f>(308411+14937+5045)/1000</f>
-        <v>328.39299999999997</v>
+        <v>1.6</v>
       </c>
       <c r="G27">
         <v>2025</v>
@@ -1873,14 +1898,13 @@
         <v>2035</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="2">
-        <f>((1307+16685)+(135+6342))*0.01163</f>
-        <v>284.57447000000002</v>
+        <v>0</v>
       </c>
       <c r="G28" t="s">
         <v>4</v>
@@ -1924,17 +1948,16 @@
     </row>
     <row r="29" spans="1:37" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D29" s="2">
-        <f>15/3.6</f>
-        <v>4.166666666666667</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="G29" t="s">
         <v>11</v>
@@ -1982,16 +2005,16 @@
     </row>
     <row r="30" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D30" s="2">
-        <v>1.07</v>
+        <v>49.879769289999999</v>
       </c>
       <c r="G30" t="s">
         <v>9</v>
@@ -2026,16 +2049,16 @@
     </row>
     <row r="31" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D31" s="2">
-        <v>0</v>
+        <v>58.785076179999997</v>
       </c>
       <c r="L31" s="4"/>
       <c r="M31" s="4"/>
@@ -2057,17 +2080,16 @@
     </row>
     <row r="32" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D32" s="2">
-        <f>26076.37044/1000</f>
-        <v>26.076370439999998</v>
+        <v>295.84986863</v>
       </c>
       <c r="G32" t="s">
         <v>38</v>
@@ -2104,17 +2126,16 @@
     </row>
     <row r="33" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D33" s="2">
-        <f>98919.26038/1000</f>
-        <v>98.919260380000011</v>
+        <v>1.958</v>
       </c>
       <c r="G33" t="s">
         <v>37</v>
@@ -2154,17 +2175,16 @@
     </row>
     <row r="34" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D34" s="2">
-        <f>(125394.01788+38683.81774)/1000</f>
-        <v>164.07783562</v>
+        <v>515.07386619106285</v>
       </c>
       <c r="H34" s="4"/>
       <c r="I34" s="4"/>
@@ -2199,17 +2219,16 @@
     </row>
     <row r="35" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D35" s="2">
-        <f>30713.3540662041*0.01163</f>
-        <v>357.19630778995366</v>
+        <v>328.39299999999997</v>
       </c>
       <c r="H35" s="4"/>
       <c r="I35" s="4"/>
@@ -2244,17 +2263,16 @@
     </row>
     <row r="36" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D36" s="2">
-        <f>(246827+6065+159)/1000</f>
-        <v>253.05099999999999</v>
+        <v>267.80401000000001</v>
       </c>
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
@@ -2289,17 +2307,16 @@
     </row>
     <row r="37" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="D37" s="2">
-        <f>((762+4941)+(96+1713))*0.01163</f>
-        <v>87.364559999999997</v>
+        <v>69.453543160961488</v>
       </c>
       <c r="L37" s="4"/>
       <c r="M37" s="4"/>
@@ -2330,7 +2347,7 @@
     </row>
     <row r="38" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>4</v>
@@ -2339,7 +2356,6 @@
         <v>5</v>
       </c>
       <c r="D38" s="2">
-        <f>15/3.6</f>
         <v>4.166666666666667</v>
       </c>
       <c r="L38" s="4"/>
@@ -2371,7 +2387,7 @@
     </row>
     <row r="39" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>4</v>
@@ -2380,7 +2396,7 @@
         <v>6</v>
       </c>
       <c r="D39" s="2">
-        <v>0.53</v>
+        <v>1.07</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="4"/>
@@ -2411,7 +2427,7 @@
     </row>
     <row r="40" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>4</v>
@@ -2455,17 +2471,16 @@
     </row>
     <row r="41" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D41" s="2">
-        <f>17885.7163/1000</f>
-        <v>17.885716299999999</v>
+        <v>3.8888888888888888</v>
       </c>
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
@@ -2500,17 +2515,16 @@
     </row>
     <row r="42" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D42" s="2">
-        <f>105580.62756/1000</f>
-        <v>105.58062756</v>
+        <v>26.076370439999998</v>
       </c>
       <c r="G42" t="s">
         <v>40</v>
@@ -2548,17 +2562,16 @@
     </row>
     <row r="43" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D43" s="2">
-        <f>(44374.63135+17534.83069)/1000</f>
-        <v>61.909462040000001</v>
+        <v>98.919260380000011</v>
       </c>
       <c r="G43" t="s">
         <v>30</v>
@@ -2636,17 +2649,16 @@
     </row>
     <row r="44" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D44" s="2">
-        <f>22877.2405523608*0.01163</f>
-        <v>266.06230762395609</v>
+        <v>164.07783562</v>
       </c>
       <c r="G44" s="13" t="s">
         <v>14</v>
@@ -2724,17 +2736,16 @@
     </row>
     <row r="45" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="D45" s="2">
-        <f>(191342+2597+14)/1000</f>
-        <v>193.953</v>
+        <v>2.1139770800000002</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
@@ -2769,17 +2780,16 @@
     </row>
     <row r="46" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D46" s="2">
-        <f>((683+4708)+(119+3092))*0.01163</f>
-        <v>100.04125999999999</v>
+        <v>357.19630778995366</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
@@ -2814,17 +2824,16 @@
     </row>
     <row r="47" spans="1:37" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
-        <v>2050</v>
+        <v>2040</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D47" s="2">
-        <f>15/3.6</f>
-        <v>4.166666666666667</v>
+        <v>253.05099999999999</v>
       </c>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
@@ -2859,16 +2868,16 @@
     </row>
     <row r="48" spans="1:37" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
-        <v>2050</v>
+        <v>2040</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D48" s="2">
-        <v>0</v>
+        <v>77.386020000000002</v>
       </c>
       <c r="L48" s="16">
         <v>2024</v>
@@ -2892,16 +2901,16 @@
     </row>
     <row r="49" spans="1:28" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
-        <v>2050</v>
+        <v>2040</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="D49" s="2">
-        <v>0</v>
+        <v>42.180018557199688</v>
       </c>
       <c r="L49" s="19"/>
       <c r="M49" s="20" t="s">
@@ -2931,17 +2940,16 @@
     </row>
     <row r="50" spans="1:28" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D50" s="2">
-        <f>11139.91081/1000</f>
-        <v>11.13991081</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="L50" s="22" t="s">
         <v>4</v>
@@ -2955,149 +2963,333 @@
     </row>
     <row r="51" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="2">
-        <f>99944.06764/1000</f>
-        <v>99.94406764</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="52" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="2">
-        <f>(2795.9212+0)/1000</f>
-        <v>2.7959212000000004</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D53" s="2">
-        <f>22264.1812466456*0.01163</f>
-        <v>258.9324278984883</v>
+        <v>3.6111111111111112</v>
       </c>
     </row>
     <row r="54" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D54" s="2">
-        <f>(183101+1374+7)/1000</f>
-        <v>184.482</v>
+        <v>17.885716299999999</v>
       </c>
     </row>
     <row r="55" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55" s="2">
+        <v>105.58062756</v>
+      </c>
+    </row>
+    <row r="56" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="2">
+        <v>61.909462040000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A57" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D57" s="2">
+        <v>1.2574564800000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58" s="2">
+        <v>266.06230762395609</v>
+      </c>
+    </row>
+    <row r="59" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D59" s="2">
+        <v>193.953</v>
+      </c>
+      <c r="E59" s="1"/>
+    </row>
+    <row r="60" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="2">
+        <v>90.713999999999999</v>
+      </c>
+      <c r="M60" s="2"/>
+    </row>
+    <row r="61" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D61" s="2">
+        <v>20.6226571890139</v>
+      </c>
+      <c r="M61" s="2"/>
+    </row>
+    <row r="62" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
         <v>2050</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C55" s="3" t="s">
+      <c r="B62" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" s="2">
+        <v>4.166666666666667</v>
+      </c>
+      <c r="M62" s="2"/>
+    </row>
+    <row r="63" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" s="2">
+        <v>0</v>
+      </c>
+      <c r="M63" s="2"/>
+    </row>
+    <row r="64" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D55" s="2">
-        <f>((560+4085)+(106+3819))*0.01163</f>
-        <v>99.6691</v>
-      </c>
-    </row>
-    <row r="56" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-    </row>
-    <row r="57" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-    </row>
-    <row r="58" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-    </row>
-    <row r="59" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-    </row>
-    <row r="60" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A60" s="2"/>
-      <c r="M60" s="2"/>
-    </row>
-    <row r="61" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A61" s="2"/>
-      <c r="M61" s="2"/>
-    </row>
-    <row r="62" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A62" s="2"/>
-      <c r="M62" s="2"/>
-    </row>
-    <row r="63" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A63" s="2"/>
-      <c r="M63" s="2"/>
-    </row>
-    <row r="64" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A64" s="2"/>
+      <c r="D64" s="2">
+        <v>0</v>
+      </c>
       <c r="M64" s="2"/>
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A65" s="2"/>
+      <c r="A65" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D65" s="2">
+        <v>3.333333333333333</v>
+      </c>
       <c r="M65" s="2"/>
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A66" s="2"/>
+      <c r="A66" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" s="2">
+        <v>11.13991081</v>
+      </c>
       <c r="M66" s="2"/>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A67" s="2"/>
+      <c r="A67" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D67" s="2">
+        <v>99.94406764</v>
+      </c>
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A68" s="2"/>
+      <c r="A68" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="2">
+        <v>2.7959212000000004</v>
+      </c>
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A69" s="2"/>
+      <c r="A69" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A70" s="2"/>
+      <c r="A70" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D70" s="2">
+        <v>258.9324278984883</v>
+      </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A71" s="2"/>
+      <c r="A71" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D71" s="2">
+        <v>184.482</v>
+      </c>
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A72" s="2"/>
+      <c r="A72" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D72" s="2">
+        <v>91.923519999999996</v>
+      </c>
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A73" s="2"/>
+      <c r="A73" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73" s="2">
+        <v>12.692282541486639</v>
+      </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
@@ -3884,7 +4076,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3731AADC-16E5-4322-A027-AF430F4F8492}">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3902,7 +4094,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2">
         <v>2026</v>
       </c>
       <c r="B2" t="s">
@@ -3912,12 +4104,11 @@
         <v>5</v>
       </c>
       <c r="D2" s="2">
-        <f>28/3.6</f>
         <v>7.7777777777777777</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="A3">
         <v>2026</v>
       </c>
       <c r="B3" t="s">
@@ -3927,12 +4118,11 @@
         <v>6</v>
       </c>
       <c r="D3" s="2">
-        <f>2.67</f>
         <v>2.67</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+      <c r="A4">
         <v>2026</v>
       </c>
       <c r="B4" t="s">
@@ -3942,502 +4132,474 @@
         <v>7</v>
       </c>
       <c r="D4" s="2">
-        <f>(27+10)/1000</f>
         <v>3.6999999999999998E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="A5">
         <v>2026</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D5" s="2">
-        <f>108002.01194/1000</f>
-        <v>108.00201194</v>
+        <v>1.1111111111111112</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="A6">
         <v>2026</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6" s="2">
-        <f>92367.37174/1000</f>
-        <v>92.367371739999996</v>
+        <v>68.366</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="A7">
         <v>2026</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2">
+        <v>192.197</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>2026</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="2">
-        <f>(306984.86711+84484.70625)/1000</f>
-        <v>391.46957335999997</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="D8" s="2">
+        <v>346.64400000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
         <v>2026</v>
       </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2.113</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>2026</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="2">
-        <f>76029.7465155539*0.01163</f>
+      <c r="D10" s="2">
         <v>884.2259519758918</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
         <v>2026</v>
       </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="2">
-        <f>(512731.305090136+32085+13246)/1000</f>
+      <c r="D11" s="2">
         <v>558.06230509013596</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>2026</v>
       </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="2">
-        <f>((4779+64753)+(1341+33309))*0.01163</f>
-        <v>1211.6366599999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+      <c r="D12" s="2">
+        <v>1140.4610599999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>2026</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="2">
+        <v>37.147113297707328</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>2030</v>
       </c>
-      <c r="B11" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="2">
-        <f>21.5/3.6</f>
-        <v>5.9722222222222223</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
-        <v>2030</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" s="2">
-        <v>2.14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
-        <v>2030</v>
-      </c>
-      <c r="B13" t="s">
-        <v>4</v>
-      </c>
-      <c r="C13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
-        <v>2030</v>
-      </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C14" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="2">
-        <f>83808.51264/1000</f>
-        <v>83.808512640000004</v>
+        <v>5.9722222222222223</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+      <c r="A15">
         <v>2030</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C15" t="s">
         <v>6</v>
       </c>
       <c r="D15" s="2">
-        <f>59066.88433/1000</f>
-        <v>59.066884330000001</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+      <c r="A16">
         <v>2030</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C16" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="2">
-        <f>(304612.30516+74920.18644)/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>2030</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="2">
+        <v>2.2222222222222223</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>2030</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2">
+        <v>83.808512640000004</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>2030</v>
+      </c>
+      <c r="B19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" s="2">
+        <v>59.066884330000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>2030</v>
+      </c>
+      <c r="B20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="2">
         <v>379.53249160000001</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>2030</v>
       </c>
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1.2689999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>2030</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
         <v>5</v>
       </c>
-      <c r="D17" s="2">
-        <f>59349.0264746045*0.01163</f>
+      <c r="D22" s="2">
         <v>690.22917789965027</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>2030</v>
       </c>
-      <c r="B18" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="2">
-        <f>(436539+21487+8798)/1000</f>
+      <c r="D23" s="2">
         <v>466.82400000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>2030</v>
       </c>
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="2">
-        <f>((2365+38938)+(561+17215))*0.01163</f>
-        <v>687.08876999999995</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="26">
+      <c r="D24" s="2">
+        <v>653.05939000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>2030</v>
+      </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="2">
+        <v>70.128610870803428</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
         <v>2035</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="2">
-        <f>15/3.6</f>
-        <v>4.166666666666667</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="26">
-        <v>2035</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="2">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="26">
-        <v>2035</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="26">
-        <v>2035</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="2">
-        <f>49879.76929/1000</f>
-        <v>49.879769289999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="26">
-        <v>2035</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" s="2">
-        <f>58785.07618/1000</f>
-        <v>58.785076179999997</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="26">
-        <v>2035</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="2">
-        <f>(231931.47942+63918.38921)/1000</f>
-        <v>295.84986863</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="26">
-        <v>2035</v>
-      </c>
       <c r="B26" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D26" s="2">
-        <f>44288.3805839263*0.01163</f>
-        <v>515.07386619106285</v>
+        <v>4.166666666666667</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="26">
+      <c r="A27" s="3">
         <v>2035</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="2">
-        <f>(308411+14937+5045)/1000</f>
-        <v>328.39299999999997</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="26">
+      <c r="A28" s="3">
         <v>2035</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D28" s="2">
-        <f>((1307+16685)+(135+6342))*0.01163</f>
-        <v>284.57447000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="26">
-        <v>2040</v>
+      <c r="A29" s="3">
+        <v>2035</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="2">
+        <v>3.333333333333333</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="2">
-        <f>15/3.6</f>
-        <v>4.166666666666667</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="26">
-        <v>2040</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="D30" s="2">
+        <v>49.879769289999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D30" s="2">
-        <v>1.07</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="26">
-        <v>2040</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>7</v>
-      </c>
       <c r="D31" s="2">
-        <v>0</v>
+        <v>58.785076179999997</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="26">
-        <v>2040</v>
+      <c r="A32" s="3">
+        <v>2035</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="2">
+        <v>295.84986863</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="2">
+        <v>1.958</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D32" s="2">
-        <f>26076.37044/1000</f>
-        <v>26.076370439999998</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="26">
+      <c r="D34" s="2">
+        <v>515.07386619106285</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="2">
+        <v>328.39299999999997</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="2">
+        <v>267.80401000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="3">
+        <v>2035</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37" s="2">
+        <v>69.453543160961488</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="3">
         <v>2040</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="2">
-        <f>98919.26038/1000</f>
-        <v>98.919260380000011</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="26">
-        <v>2040</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="2">
-        <f>(125394.01788+38683.81774)/1000</f>
-        <v>164.07783562</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="26">
-        <v>2040</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="2">
-        <f>30713.3540662041*0.01163</f>
-        <v>357.19630778995366</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="26">
-        <v>2040</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" s="2">
-        <f>(246827+6065+159)/1000</f>
-        <v>253.05099999999999</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="26">
-        <v>2040</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="2">
-        <f>((762+4941)+(96+1713))*0.01163</f>
-        <v>87.364559999999997</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="26">
-        <v>2045</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>4</v>
@@ -4446,13 +4608,12 @@
         <v>5</v>
       </c>
       <c r="D38" s="2">
-        <f>15/3.6</f>
         <v>4.166666666666667</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="26">
-        <v>2045</v>
+      <c r="A39" s="3">
+        <v>2040</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>4</v>
@@ -4461,12 +4622,12 @@
         <v>6</v>
       </c>
       <c r="D39" s="2">
-        <v>0.53</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="26">
-        <v>2045</v>
+      <c r="A40" s="3">
+        <v>2040</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>4</v>
@@ -4479,226 +4640,465 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="26">
-        <v>2045</v>
+      <c r="A41" s="3">
+        <v>2040</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="D41" s="2">
-        <f>17885.7163/1000</f>
-        <v>17.885716299999999</v>
+        <v>3.8888888888888888</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="26">
-        <v>2045</v>
+      <c r="A42" s="3">
+        <v>2040</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D42" s="2">
-        <f>105580.62756/1000</f>
-        <v>105.58062756</v>
+        <v>26.076370439999998</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="26">
-        <v>2045</v>
+      <c r="A43" s="3">
+        <v>2040</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="2">
+        <v>98.919260380000011</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="3">
+        <v>2040</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D43" s="2">
-        <f>(44374.63135+17534.83069)/1000</f>
-        <v>61.909462040000001</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="26">
+      <c r="D44" s="2">
+        <v>164.07783562</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="3">
+        <v>2040</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D45" s="2">
+        <v>2.1139770800000002</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="3">
+        <v>2040</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D46" s="2">
+        <v>357.19630778995366</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="3">
+        <v>2040</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="2">
+        <v>253.05099999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="3">
+        <v>2040</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D48" s="2">
+        <v>77.386020000000002</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="3">
+        <v>2040</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D49" s="2">
+        <v>42.180018557199688</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50" s="3">
         <v>2045</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D44" s="2">
-        <f>22877.2405523608*0.01163</f>
-        <v>266.06230762395609</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="26">
-        <v>2045</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="2">
-        <f>(191342+2597+14)/1000</f>
-        <v>193.953</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="26">
-        <v>2045</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D46" s="2">
-        <f>((683+4708)+(119+3092))*0.01163</f>
-        <v>100.04125999999999</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="26">
-        <v>2050</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D47" s="2">
-        <f>15/3.6</f>
-        <v>4.166666666666667</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="26">
-        <v>2050</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="26">
-        <v>2050</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D49" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="26">
-        <v>2050</v>
-      </c>
       <c r="B50" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C50" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D50" s="2">
-        <f>11139.91081/1000</f>
-        <v>11.13991081</v>
+        <v>4.166666666666667</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="26">
-        <v>2050</v>
+      <c r="A51" s="3">
+        <v>2045</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D51" s="2">
-        <f>99944.06764/1000</f>
-        <v>99.94406764</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="26">
-        <v>2050</v>
+      <c r="A52" s="3">
+        <v>2045</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D52" s="2">
-        <f>(2795.9212+0)/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D53" s="2">
+        <v>3.6111111111111112</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D54" s="2">
+        <v>17.885716299999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55" s="2">
+        <v>105.58062756</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D56" s="2">
+        <v>61.909462040000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D57" s="2">
+        <v>1.2574564800000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58" s="2">
+        <v>266.06230762395609</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D59" s="2">
+        <v>193.953</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D60" s="2">
+        <v>90.713999999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="3">
+        <v>2045</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D61" s="2">
+        <v>20.6226571890139</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D62" s="2">
+        <v>4.166666666666667</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D64" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D65" s="2">
+        <v>3.333333333333333</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D66" s="2">
+        <v>11.13991081</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D67" s="2">
+        <v>99.94406764</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D68" s="2">
         <v>2.7959212000000004</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="26">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69" s="3">
         <v>2050</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C53" s="3" t="s">
+      <c r="B69" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D69" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D53" s="2">
-        <f>22264.1812466456*0.01163</f>
+      <c r="D70" s="2">
         <v>258.9324278984883</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="26">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71" s="3">
         <v>2050</v>
       </c>
-      <c r="B54" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C54" s="3" t="s">
+      <c r="B71" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D54" s="2">
-        <f>(183101+1374+7)/1000</f>
+      <c r="D71" s="2">
         <v>184.482</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="26">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72" s="3">
         <v>2050</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C55" s="3" t="s">
+      <c r="B72" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D55" s="2">
-        <f>((560+4085)+(106+3819))*0.01163</f>
-        <v>99.6691</v>
+      <c r="D72" s="2">
+        <v>91.923519999999996</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73" s="3">
+        <v>2050</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D73" s="2">
+        <v>12.692282541486639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
working model with scenarios for sens
</commit_message>
<xml_diff>
--- a/NG_flows_scm.xlsx
+++ b/NG_flows_scm.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5611d695511771a1/Desktop/Repositories/scm_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{063E1CBA-981A-4F9C-9ABC-D9966DC7B63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E77FD392-8979-4E08-976D-874911313D3A}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{063E1CBA-981A-4F9C-9ABC-D9966DC7B63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96F35781-E36A-4300-B3FD-EC976D92EEDF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{3FD26122-B3FE-4856-AD14-3A87BCC0C804}"/>
+    <workbookView xWindow="-28920" yWindow="6825" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{3FD26122-B3FE-4856-AD14-3A87BCC0C804}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="supply_share" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">demand!$C$1:$C$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$B$1:$B$275</definedName>
     <definedName name="demand_table">Tabelle1!$A$1:$D$55</definedName>
     <definedName name="supply_share">Tabelle1!$K$59:$M$66</definedName>
@@ -4196,7 +4197,7 @@
         <v>2026</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
         <v>43</v>
@@ -4364,7 +4365,7 @@
         <v>2030</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C21" t="s">
         <v>43</v>
@@ -4532,7 +4533,7 @@
         <v>2035</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>43</v>
@@ -4700,7 +4701,7 @@
         <v>2040</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>43</v>
@@ -4868,7 +4869,7 @@
         <v>2045</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>43</v>
@@ -5036,7 +5037,7 @@
         <v>2050</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>43</v>

</xml_diff>